<commit_message>
Arreglado conteo de habitaciones.
</commit_message>
<xml_diff>
--- a/room_list.xlsx
+++ b/room_list.xlsx
@@ -526,22 +526,22 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -561,10 +561,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -573,10 +573,10 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -592,22 +592,22 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5"/>
@@ -725,7 +725,7 @@
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>Single F</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>SINGLE F</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>SINGLE F</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -1825,12 +1825,12 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>BISHT</t>
+          <t>MACAPOBRE</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> LALIT</t>
+          <t xml:space="preserve"> HOMBRE</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1840,12 +1840,12 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>Service Assistant</t>
+          <t>Able Seaman</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t xml:space="preserve">Doble </t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">KALIM </t>
+          <t>BISHT</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MAZHAR</t>
+          <t xml:space="preserve"> LALIT</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Butler</t>
+          <t>Service Assistant</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -1925,7 +1925,7 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>SAHA</t>
+          <t xml:space="preserve">KALIM </t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SOUVIK</t>
+          <t xml:space="preserve"> MAZHAR</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>Suite Attendant</t>
+          <t>Butler</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="K29" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>VELANKOVIL RAJU</t>
+          <t>SAHA</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RENJITH MON</t>
+          <t xml:space="preserve"> SOUVIK</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Galley Utility</t>
+          <t>Suite Attendant</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="K30" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
@@ -2065,12 +2065,12 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>NYARIKI</t>
+          <t>VELANKOVIL RAJU</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MARTIN</t>
+          <t xml:space="preserve"> RENJITH MON</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>2nd Cook</t>
+          <t>Galley Utility</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="K31" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
@@ -2125,12 +2125,12 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>OWIYO</t>
+          <t>NYARIKI</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ERICK ODONGO</t>
+          <t xml:space="preserve"> MARTIN</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
@@ -2145,7 +2145,7 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Bartender</t>
+          <t>2nd Cook</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
@@ -2160,12 +2160,12 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>2024-11-15</t>
+          <t>2024-11-16</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
@@ -2185,12 +2185,12 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>AGUSTIN</t>
+          <t>OWIYO</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GARRY</t>
+          <t xml:space="preserve"> ERICK ODONGO</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -2200,12 +2200,12 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>2nd Cook</t>
+          <t>Bartender</t>
         </is>
       </c>
       <c r="H33" s="4" t="inlineStr">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="J33" s="4" t="inlineStr">
         <is>
-          <t>2024-11-16</t>
+          <t>2024-11-15</t>
         </is>
       </c>
       <c r="K33" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
@@ -2245,12 +2245,12 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>AREVALO</t>
+          <t>AGUSTIN</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> TIMOTEO JR. BARNES</t>
+          <t xml:space="preserve"> GARRY</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Carpenter</t>
+          <t>2nd Cook</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
@@ -2285,7 +2285,7 @@
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
@@ -2305,12 +2305,12 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>BARLAAN</t>
+          <t>AREVALO</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MARLON</t>
+          <t xml:space="preserve"> TIMOTEO JR. BARNES</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>Chef De Partie</t>
+          <t>Carpenter</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="K35" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
@@ -2365,12 +2365,12 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>CASTILLON</t>
+          <t>BARLAAN</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JOLLY PANTORILLA</t>
+          <t xml:space="preserve"> MARLON</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Able Seaman</t>
+          <t>Chef De Partie</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="K36" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
@@ -2425,12 +2425,12 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>LAURENTE</t>
+          <t>CASTILLON</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> REYMARK</t>
+          <t xml:space="preserve"> JOLLY PANTORILLA</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -2460,12 +2460,12 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>2024-11-15</t>
+          <t>2024-11-16</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
@@ -2485,12 +2485,12 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>MACAPOBRE</t>
+          <t>LAURENTE</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> HOMBRE</t>
+          <t xml:space="preserve"> REYMARK</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -2520,12 +2520,12 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>2024-11-16</t>
+          <t>2024-11-15</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="K39" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L40" s="4" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="K41" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="K42" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="K43" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L43" s="4" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="K44" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="K45" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L45" s="4" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="K46" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L46" s="4" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="K47" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L47" s="4" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="K48" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L48" s="4" t="inlineStr">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="K49" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L49" s="4" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L50" s="4" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="K51" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L51" s="4" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="K52" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L52" s="4" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="K53" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L53" s="4" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="K54" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L54" s="4" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="K55" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L55" s="4" t="inlineStr">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="K56" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L56" s="4" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="K57" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L57" s="4" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="K58" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L58" s="4" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="K59" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L59" s="4" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="K60" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L60" s="4" t="inlineStr">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="K61" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L61" s="4" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="K62" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L62" s="4" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="K63" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L63" s="4" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="K64" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L64" s="4" t="inlineStr">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="K65" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L65" s="4" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="K66" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L66" s="4" t="inlineStr">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="K67" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L67" s="4" t="inlineStr">
@@ -4285,12 +4285,12 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PHANI</t>
+          <t xml:space="preserve"> RODNEY</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>ANUMUKONDA</t>
+          <t>SENO</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
@@ -4300,12 +4300,12 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>Butler</t>
+          <t>Suite Attendant</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
@@ -4320,7 +4320,7 @@
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-11-19</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">
@@ -4345,12 +4345,12 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> KIRTI KUMAR</t>
+          <t xml:space="preserve"> PHANI</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>JENA</t>
+          <t>ANUMUKONDA</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
@@ -4365,7 +4365,7 @@
       </c>
       <c r="G69" s="4" t="inlineStr">
         <is>
-          <t>Service Assistant</t>
+          <t>Butler</t>
         </is>
       </c>
       <c r="H69" s="4" t="inlineStr">
@@ -4385,7 +4385,7 @@
       </c>
       <c r="K69" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L69" s="4" t="inlineStr">
@@ -4405,12 +4405,12 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> DEEPAK</t>
+          <t xml:space="preserve"> KIRTI KUMAR</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>KESHTWAL</t>
+          <t>JENA</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>Butler</t>
+          <t>Service Assistant</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="K70" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L70" s="4" t="inlineStr">
@@ -4465,12 +4465,12 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SAGAR </t>
+          <t xml:space="preserve"> DEEPAK</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNU </t>
+          <t>KESHTWAL</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="K71" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L71" s="4" t="inlineStr">
@@ -4525,12 +4525,12 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NANDLAL</t>
+          <t xml:space="preserve"> SAGAR </t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>RAJBHAR</t>
+          <t xml:space="preserve">LNU </t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Galley Utility</t>
+          <t>Butler</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
@@ -4560,12 +4560,12 @@
       </c>
       <c r="J72" s="4" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="K72" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L72" s="4" t="inlineStr">
@@ -4585,12 +4585,12 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> LAIJU</t>
+          <t xml:space="preserve"> NANDLAL</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>THOMAS</t>
+          <t>RAJBHAR</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
@@ -4605,7 +4605,7 @@
       </c>
       <c r="G73" s="4" t="inlineStr">
         <is>
-          <t>Chef De Partie</t>
+          <t>Galley Utility</t>
         </is>
       </c>
       <c r="H73" s="4" t="inlineStr">
@@ -4620,12 +4620,12 @@
       </c>
       <c r="J73" s="4" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-11-19</t>
         </is>
       </c>
       <c r="K73" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L73" s="4" t="inlineStr">
@@ -4645,12 +4645,12 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> I GUSTI NGURAH BAGUS</t>
+          <t xml:space="preserve"> LAIJU</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>SUADNYA</t>
+          <t>THOMAS</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
@@ -4660,12 +4660,12 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Bartender</t>
+          <t>Chef De Partie</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="J74" s="4" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="K74" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L74" s="4" t="inlineStr">
@@ -4705,12 +4705,12 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FNU</t>
+          <t xml:space="preserve"> I GUSTI NGURAH BAGUS</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>TEGUH</t>
+          <t>SUADNYA</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>Laundry Man</t>
+          <t>Bartender</t>
         </is>
       </c>
       <c r="H75" s="4" t="inlineStr">
@@ -4740,12 +4740,12 @@
       </c>
       <c r="J75" s="4" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-11-19</t>
         </is>
       </c>
       <c r="K75" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L75" s="4" t="inlineStr">
@@ -4765,12 +4765,12 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ROBIN NICENO</t>
+          <t xml:space="preserve"> FNU</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>ALABASTRO</t>
+          <t>TEGUH</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
@@ -4780,12 +4780,12 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Junior Nurse</t>
+          <t>Laundry Man</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="K76" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L76" s="4" t="inlineStr">
@@ -4825,12 +4825,12 @@
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> DANTE</t>
+          <t xml:space="preserve"> ROBIN NICENO</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>ASEOCHE</t>
+          <t>ALABASTRO</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="G77" s="4" t="inlineStr">
         <is>
-          <t>2nd Cook</t>
+          <t>Junior Nurse</t>
         </is>
       </c>
       <c r="H77" s="4" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="K77" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L77" s="4" t="inlineStr">
@@ -4885,12 +4885,12 @@
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JONATHAN</t>
+          <t xml:space="preserve"> DANTE</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>BALANCIO</t>
+          <t>ASEOCHE</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -4905,7 +4905,7 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Able Seaman</t>
+          <t>2nd Cook</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
@@ -4925,7 +4925,7 @@
       </c>
       <c r="K78" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L78" s="4" t="inlineStr">
@@ -4945,12 +4945,12 @@
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RONNIE GIDOR</t>
+          <t xml:space="preserve"> JONATHAN</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>BALLINAS</t>
+          <t>BALANCIO</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="G79" s="4" t="inlineStr">
         <is>
-          <t>Fitter</t>
+          <t>Able Seaman</t>
         </is>
       </c>
       <c r="H79" s="4" t="inlineStr">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="K79" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L79" s="4" t="inlineStr">
@@ -5005,12 +5005,12 @@
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ERMIE</t>
+          <t xml:space="preserve"> RONNIE GIDOR</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>CARINO</t>
+          <t>BALLINAS</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -5025,7 +5025,7 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Chef De Partie</t>
+          <t>Fitter</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="K80" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L80" s="4" t="inlineStr">
@@ -5065,12 +5065,12 @@
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> WILLIAM</t>
+          <t xml:space="preserve"> ERMIE</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>DOLLENTAS</t>
+          <t>CARINO</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="G81" s="4" t="inlineStr">
         <is>
-          <t>Chef De Cuisine</t>
+          <t>Chef De Partie</t>
         </is>
       </c>
       <c r="H81" s="4" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="K81" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L81" s="4" t="inlineStr">
@@ -5125,12 +5125,12 @@
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JERUH FULAY</t>
+          <t xml:space="preserve"> WILLIAM</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>FLORIDA</t>
+          <t>DOLLENTAS</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>Carpenter</t>
+          <t>Chef De Cuisine</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="K82" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L82" s="4" t="inlineStr">
@@ -5185,12 +5185,12 @@
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ERIK MARIONNE MANUIT</t>
+          <t xml:space="preserve"> JERUH FULAY</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>JATULAN</t>
+          <t>FLORIDA</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="G83" s="4" t="inlineStr">
         <is>
-          <t>Galley Utility</t>
+          <t>Carpenter</t>
         </is>
       </c>
       <c r="H83" s="4" t="inlineStr">
@@ -5220,12 +5220,12 @@
       </c>
       <c r="J83" s="4" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="K83" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L83" s="4" t="inlineStr">
@@ -5245,12 +5245,12 @@
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JUSTIN HANNS ORTIZO</t>
+          <t xml:space="preserve"> ERIK MARIONNE MANUIT</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>LANIOG</t>
+          <t>JATULAN</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
@@ -5265,7 +5265,7 @@
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Desktop Publisher</t>
+          <t>Galley Utility</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="K84" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L84" s="4" t="inlineStr">
@@ -5305,12 +5305,12 @@
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> EDUARD FLORES</t>
+          <t xml:space="preserve"> JUSTIN HANNS ORTIZO</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>MARIKIT</t>
+          <t>LANIOG</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="G85" s="4" t="inlineStr">
         <is>
-          <t>Able Seaman</t>
+          <t>Desktop Publisher</t>
         </is>
       </c>
       <c r="H85" s="4" t="inlineStr">
@@ -5340,12 +5340,12 @@
       </c>
       <c r="J85" s="4" t="inlineStr">
         <is>
-          <t>2024-11-18</t>
+          <t>2024-11-19</t>
         </is>
       </c>
       <c r="K85" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L85" s="4" t="inlineStr">
@@ -5365,12 +5365,12 @@
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GEM LASKER ARCELO</t>
+          <t xml:space="preserve"> EDUARD FLORES</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>PURIO</t>
+          <t>MARIKIT</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>Provision Man</t>
+          <t>Able Seaman</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="K86" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L86" s="4" t="inlineStr">
@@ -5425,12 +5425,12 @@
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RODNEY</t>
+          <t xml:space="preserve"> GEM LASKER ARCELO</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>SENO</t>
+          <t>PURIO</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -5445,7 +5445,7 @@
       </c>
       <c r="G87" s="4" t="inlineStr">
         <is>
-          <t>Suite Attendant</t>
+          <t>Provision Man</t>
         </is>
       </c>
       <c r="H87" s="4" t="inlineStr">
@@ -5460,12 +5460,12 @@
       </c>
       <c r="J87" s="4" t="inlineStr">
         <is>
-          <t>2024-11-19</t>
+          <t>2024-11-18</t>
         </is>
       </c>
       <c r="K87" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L87" s="4" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="K89" s="4" t="inlineStr">
         <is>
-          <t>Doble F</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L89" s="4" t="inlineStr">
@@ -5605,12 +5605,12 @@
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RIZWAN</t>
+          <t xml:space="preserve"> ALCIDES IVAN</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>SHAGUL HAMEED</t>
+          <t>PONTE VARA</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -5620,12 +5620,12 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>Executive Sous Chef</t>
+          <t>IT/Communications Officer</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
@@ -5645,7 +5645,7 @@
       </c>
       <c r="K90" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L90" s="4" t="inlineStr">
@@ -5665,12 +5665,12 @@
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ALCIDES IVAN</t>
+          <t xml:space="preserve"> NORBERTO</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>PONTE VARA</t>
+          <t>OXENO</t>
         </is>
       </c>
       <c r="E91" s="4" t="inlineStr">
@@ -5680,12 +5680,12 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="G91" s="4" t="inlineStr">
         <is>
-          <t>IT/Communications Officer</t>
+          <t>Head Bartender</t>
         </is>
       </c>
       <c r="H91" s="4" t="inlineStr">
@@ -5705,7 +5705,7 @@
       </c>
       <c r="K91" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Single</t>
         </is>
       </c>
       <c r="L91" s="4" t="inlineStr">
@@ -5725,12 +5725,12 @@
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NORBERTO</t>
+          <t xml:space="preserve"> PHANI</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>OXENO</t>
+          <t>ANUMUKONDA</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -5740,12 +5740,12 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Head Bartender</t>
+          <t>Butler</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
@@ -5765,12 +5765,12 @@
       </c>
       <c r="K92" s="4" t="inlineStr">
         <is>
-          <t>Single M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L92" s="4" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AW</t>
         </is>
       </c>
     </row>
@@ -5785,12 +5785,12 @@
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> PHANI</t>
+          <t xml:space="preserve"> KIRTI KUMAR</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>ANUMUKONDA</t>
+          <t>JENA</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="G93" s="4" t="inlineStr">
         <is>
-          <t>Butler</t>
+          <t>Service Assistant</t>
         </is>
       </c>
       <c r="H93" s="4" t="inlineStr">
@@ -5825,12 +5825,12 @@
       </c>
       <c r="K93" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L93" s="4" t="inlineStr">
         <is>
-          <t>AW</t>
+          <t>BA</t>
         </is>
       </c>
     </row>
@@ -5845,12 +5845,12 @@
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> KIRTI KUMAR</t>
+          <t xml:space="preserve"> DEEPAK</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>JENA</t>
+          <t>KESHTWAL</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -5865,7 +5865,7 @@
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Service Assistant</t>
+          <t>Butler</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
@@ -5885,12 +5885,12 @@
       </c>
       <c r="K94" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L94" s="4" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BA</t>
         </is>
       </c>
     </row>
@@ -5905,12 +5905,12 @@
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> DEEPAK</t>
+          <t xml:space="preserve"> SAGAR </t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>KESHTWAL</t>
+          <t xml:space="preserve">LNU </t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="K95" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L95" s="4" t="inlineStr">
@@ -5965,12 +5965,12 @@
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> SAGAR </t>
+          <t xml:space="preserve"> RIZWAN</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNU </t>
+          <t>SHAGUL HAMEED</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
@@ -5985,7 +5985,7 @@
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Butler</t>
+          <t>Executive Sous Chef</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
@@ -6005,12 +6005,12 @@
       </c>
       <c r="K96" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L96" s="4" t="inlineStr">
         <is>
-          <t>BC</t>
+          <t>BB</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="K97" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L97" s="4" t="inlineStr">
@@ -6125,12 +6125,12 @@
       </c>
       <c r="K98" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L98" s="4" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>BC</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6185,7 @@
       </c>
       <c r="K99" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L99" s="4" t="inlineStr">
@@ -6245,12 +6245,12 @@
       </c>
       <c r="K100" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L100" s="4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BD</t>
         </is>
       </c>
     </row>
@@ -6305,7 +6305,7 @@
       </c>
       <c r="K101" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L101" s="4" t="inlineStr">
@@ -6365,12 +6365,12 @@
       </c>
       <c r="K102" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L102" s="4" t="inlineStr">
         <is>
-          <t>BF</t>
+          <t>BE</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6425,7 @@
       </c>
       <c r="K103" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L103" s="4" t="inlineStr">
@@ -6485,12 +6485,12 @@
       </c>
       <c r="K104" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L104" s="4" t="inlineStr">
         <is>
-          <t>BG</t>
+          <t>BF</t>
         </is>
       </c>
     </row>
@@ -6505,12 +6505,12 @@
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NANDLAL</t>
+          <t xml:space="preserve"> I GUSTI NGURAH BAGUS</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>RAJBHAR</t>
+          <t>SUADNYA</t>
         </is>
       </c>
       <c r="E105" s="4" t="inlineStr">
@@ -6520,12 +6520,12 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="G105" s="4" t="inlineStr">
         <is>
-          <t>Galley Utility</t>
+          <t>Bartender</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">
@@ -6565,12 +6565,12 @@
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> I GUSTI NGURAH BAGUS</t>
+          <t xml:space="preserve"> RODNEY</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>SUADNYA</t>
+          <t>SENO</t>
         </is>
       </c>
       <c r="E106" s="4" t="inlineStr">
@@ -6580,12 +6580,12 @@
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>Bartender</t>
+          <t>Suite Attendant</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
@@ -6610,7 +6610,7 @@
       </c>
       <c r="L106" s="4" t="inlineStr">
         <is>
-          <t>BH</t>
+          <t>BG</t>
         </is>
       </c>
     </row>
@@ -6625,12 +6625,12 @@
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ERIK MARIONNE MANUIT</t>
+          <t xml:space="preserve"> NANDLAL</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>JATULAN</t>
+          <t>RAJBHAR</t>
         </is>
       </c>
       <c r="E107" s="4" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>India</t>
         </is>
       </c>
       <c r="G107" s="4" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="K107" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L107" s="4" t="inlineStr">
@@ -6685,12 +6685,12 @@
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> JUSTIN HANNS ORTIZO</t>
+          <t xml:space="preserve"> ERIK MARIONNE MANUIT</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>LANIOG</t>
+          <t>JATULAN</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
@@ -6705,7 +6705,7 @@
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>Desktop Publisher</t>
+          <t>Galley Utility</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
@@ -6725,12 +6725,12 @@
       </c>
       <c r="K108" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L108" s="4" t="inlineStr">
         <is>
-          <t>BI</t>
+          <t>BH</t>
         </is>
       </c>
     </row>
@@ -6745,12 +6745,12 @@
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RODNEY</t>
+          <t xml:space="preserve"> JUSTIN HANNS ORTIZO</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>SENO</t>
+          <t>LANIOG</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
@@ -6765,7 +6765,7 @@
       </c>
       <c r="G109" s="4" t="inlineStr">
         <is>
-          <t>Suite Attendant</t>
+          <t>Desktop Publisher</t>
         </is>
       </c>
       <c r="H109" s="4" t="inlineStr">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="K109" s="4" t="inlineStr">
         <is>
-          <t>Doble M</t>
+          <t>Doble</t>
         </is>
       </c>
       <c r="L109" s="4" t="inlineStr">

</xml_diff>